<commit_message>
Fix: Add AWS to Cost Structure, show ,054K fixed cost derivation
</commit_message>
<xml_diff>
--- a/GC/part_b/deliverables/business_model.xlsx
+++ b/GC/part_b/deliverables/business_model.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="167" formatCode="$#,##0.000"/>
+    <numFmt numFmtId="167" formatCode="#,##0.000"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -2057,7 +2057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2571,44 +2571,55 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Annual Fixed Cost</t>
+          <t>Platform Operations (AWS)</t>
         </is>
       </c>
       <c r="B34" s="12">
-        <f>B30+B31+B32+B33</f>
+        <f>Assumptions!B59*12</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Annual Data Volume (GB)</t>
-        </is>
-      </c>
-      <c r="B35" s="14">
-        <f>5*Assumptions!B18*Assumptions!B19*365*Assumptions!B21</f>
+          <t>Annual Fixed Cost (~$1,054K at maturity)</t>
+        </is>
+      </c>
+      <c r="B35" s="12">
+        <f>B30+B31+B32+B33+B34</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cost per GB (cents)</t>
-        </is>
-      </c>
-      <c r="B36" s="15">
-        <f>B34/B35*100</f>
+          <t>Annual Data Volume (GB)</t>
+        </is>
+      </c>
+      <c r="B36" s="14">
+        <f>5*Assumptions!B18*Assumptions!B19*365*Assumptions!B21</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>Cost per GB (cents)</t>
+        </is>
+      </c>
+      <c r="B37" s="15">
+        <f>B35/B36*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>Revenue at 40% util, $1/GB</t>
         </is>
       </c>
-      <c r="B37" s="12">
-        <f>B35*0.4*Assumptions!B17</f>
+      <c r="B38" s="12">
+        <f>B36*0.4*Assumptions!B17</f>
         <v/>
       </c>
     </row>

</xml_diff>